<commit_message>
Move packaging quantities to separate Verpackung sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ebndxv7vKn8rcczFHNKhFK
</commit_message>
<xml_diff>
--- a/lager-scanner/Lager_Vorlage.xlsx
+++ b/lager-scanner/Lager_Vorlage.xlsx
@@ -8,13 +8,16 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialliste" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stellplaetze" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protokoll" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lageruebersicht" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlanLayout" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagerplan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verpackung" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stellplaetze" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protokoll" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lageruebersicht" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlanLayout" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagerplan" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Verpackung'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -190,22 +193,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblMaterial" displayName="tblMaterial" ref="A1:F2" headerRowCount="1">
-  <autoFilter ref="A1:F2"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblMaterial" displayName="tblMaterial" ref="A1:D2" headerRowCount="1">
+  <autoFilter ref="A1:D2"/>
+  <tableColumns count="4">
     <tableColumn id="1" name="SAP"/>
     <tableColumn id="2" name="Bezeichnung"/>
     <tableColumn id="3" name="Lagerstand"/>
     <tableColumn id="4" name="Meldebestand"/>
-    <tableColumn id="5" name="StkProKarton"/>
-    <tableColumn id="6" name="StkProPalette"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblStellplatz" displayName="tblStellplatz" ref="A1:B2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblVerpackung" displayName="tblVerpackung" ref="A1:D2" headerRowCount="1">
+  <autoFilter ref="A1:D2"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="SAP"/>
+    <tableColumn id="2" name="Bezeichnung"/>
+    <tableColumn id="3" name="StkProPalette"/>
+    <tableColumn id="4" name="StkProKarton"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblStellplatz" displayName="tblStellplatz" ref="A1:B2" headerRowCount="1">
   <autoFilter ref="A1:B2"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Stellplatz"/>
@@ -215,8 +229,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblProtokoll" displayName="tblProtokoll" ref="A1:H2" headerRowCount="1">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblProtokoll" displayName="tblProtokoll" ref="A1:H2" headerRowCount="1">
   <autoFilter ref="A1:H2"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Zeit"/>
@@ -521,15 +535,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,16 +565,6 @@
           <t>Meldebestand</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>StkProKarton</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>StkProPalette</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -580,12 +582,6 @@
       </c>
       <c r="D2" t="n">
         <v>10</v>
-      </c>
-      <c r="E2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F2" t="n">
-        <v>480</v>
       </c>
     </row>
   </sheetData>
@@ -597,6 +593,70 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Bezeichnung</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>StkProPalette</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>StkProKarton</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>1000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Beispielmaterial</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>480</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -635,7 +695,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -714,7 +774,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26768,7 +26828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26913,7 +26973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>